<commit_message>
Add sub-service owner fields, auto-sizing cards and parallel split decision node
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/service-catalog-template.xlsx
+++ b/public/service-catalog-template.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -576,6 +576,8 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -604,6 +606,16 @@
           <t>active</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>owner_name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>owner_email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -631,6 +643,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Fatima Al Suwaidi</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>fatima.alsuwaidi@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -658,6 +680,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Fatima Al Suwaidi</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>fatima.alsuwaidi@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -685,6 +717,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Fatima Al Suwaidi</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>fatima.alsuwaidi@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -712,6 +754,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Fatima Al Suwaidi</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>fatima.alsuwaidi@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -739,6 +791,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Fatima Al Suwaidi</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>fatima.alsuwaidi@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -766,6 +828,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Omar Hassan</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>omar.hassan@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -793,6 +865,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Omar Hassan</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>omar.hassan@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -820,6 +902,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Omar Hassan</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>omar.hassan@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -845,6 +937,16 @@
       <c r="E10" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Omar Hassan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>omar.hassan@example.com</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1611,6 +1713,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1639,6 +1742,11 @@
           <t>execution_mode</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1664,6 +1772,11 @@
           <t>PARALLEL</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1689,6 +1802,11 @@
           <t>PARALLEL</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>If laptop required</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1712,6 +1830,11 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>PARALLEL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>If on-site employee</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2626,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>the Service Request itself (the parent request); entitlement and SLA now live in their own tabs</t>
+          <t>the Service Request itself (the parent request); owner_name/owner_email are the sub-service owner; entitlement and SLA live in their own tabs</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2694,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>execution_mode = PARALLEL (all raised at once) or SEQUENCE (raised in seq order)</t>
+          <t>execution_mode = PARALLEL (all raised at once) or SEQUENCE (raised in seq order); condition = the branch rule shown on the split</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add conditional approvals: condition column plus approval decision gate and skip path
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/service-catalog-template.xlsx
+++ b/public/service-catalog-template.xlsx
@@ -1403,13 +1403,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1433,6 +1434,11 @@
           <t>approver</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1573,6 +1579,11 @@
           <t>Finance</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>If trip cost &gt; AED 10,000</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1591,6 +1602,11 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>HR Head</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>If international travel</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2693,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0 rows = auto-approved; N rows = N levels, no schema change needed</t>
+          <t>0 rows = auto-approved; N rows = N levels; condition = rule that decides whether the level applies (blank = always)</t>
         </is>
       </c>
     </row>

</xml_diff>